<commit_message>
change pc handle data
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-221af0.o</t>
+    <t>lto-llvm-8b0af1.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -240,7 +240,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-221af0.o</c:v>
+                  <c:v>lto-llvm-8b0af1.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -258,10 +258,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>92.76171875</c:v>
+                  <c:v>91.75058746337891</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.238283634185791</c:v>
+                  <c:v>8.249416351318359</c:v>
                 </c:pt>
                 <c:pt idx="33">
                   <c:v>0</c:v>
@@ -335,7 +335,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-221af0.o</c:v>
+                  <c:v>lto-llvm-8b0af1.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -446,103 +446,103 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>89.18135833740234</c:v>
+                  <c:v>89.21461486816406</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.395655632019043</c:v>
+                  <c:v>4.382145404815674</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.9435945153236389</c:v>
+                  <c:v>0.9406943321228027</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.780100405216217</c:v>
+                  <c:v>0.7777027487754822</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.5418661832809448</c:v>
+                  <c:v>0.5402007102966309</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.5325236320495606</c:v>
+                  <c:v>0.5308868885040283</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.5185098648071289</c:v>
+                  <c:v>0.5169162154197693</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4344271719455719</c:v>
+                  <c:v>0.433091938495636</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4110708832740784</c:v>
+                  <c:v>0.4098074436187744</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2896181344985962</c:v>
+                  <c:v>0.2887279689311981</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.2569192945957184</c:v>
+                  <c:v>0.256129652261734</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2335630059242249</c:v>
+                  <c:v>0.2328451275825501</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1448090672492981</c:v>
+                  <c:v>0.1443639844655991</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.1167815029621124</c:v>
+                  <c:v>0.116422563791275</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.1167815029621124</c:v>
+                  <c:v>0.116422563791275</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1121102422475815</c:v>
+                  <c:v>0.111765667796135</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.0934251993894577</c:v>
+                  <c:v>0.09313805401325226</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.08408267796039581</c:v>
+                  <c:v>0.08382424712181091</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.08408267796039581</c:v>
+                  <c:v>0.08382424712181091</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.07941142469644547</c:v>
+                  <c:v>0.07916734367609024</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.07474016398191452</c:v>
+                  <c:v>0.07451044023036957</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.07006890326738358</c:v>
+                  <c:v>0.0698535367846489</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.07006890326738358</c:v>
+                  <c:v>0.0698535367846489</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06539764255285263</c:v>
+                  <c:v>0.06519664078950882</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.06539764255285263</c:v>
+                  <c:v>0.06519664078950882</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.06539764255285263</c:v>
+                  <c:v>0.06519664078950882</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.06539764255285263</c:v>
+                  <c:v>0.06519664078950882</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.06072638183832169</c:v>
+                  <c:v>0.06053973361849785</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.04204133898019791</c:v>
+                  <c:v>0.04191212356090546</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02335629984736443</c:v>
+                  <c:v>0.02328451350331307</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01868504099547863</c:v>
+                  <c:v>0.01862761005759239</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01868504099547863</c:v>
+                  <c:v>0.01862761005759239</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.009342520497739315</c:v>
+                  <c:v>0.009313805028796196</c:v>
                 </c:pt>
                 <c:pt idx="33">
                   <c:v>0</c:v>
@@ -1009,25 +1009,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>92.76171875</v>
+        <v>91.75058746337891</v>
       </c>
       <c r="C3" s="1">
-        <v>13123</v>
+        <v>11389</v>
       </c>
       <c r="D3" s="1">
-        <v>38183</v>
+        <v>38315</v>
       </c>
       <c r="E3" s="1">
-        <v>37940</v>
+        <v>38054</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>12986</v>
+        <v>11234</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1035,7 +1035,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>7.238283634185791</v>
+        <v>8.249416351318359</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1142,25 +1142,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.18135833740234</v>
+        <v>89.21461486816406</v>
       </c>
       <c r="C3" s="1">
-        <v>38183</v>
+        <v>38315</v>
       </c>
       <c r="D3" s="1">
-        <v>13123</v>
+        <v>11389</v>
       </c>
       <c r="E3" s="1">
-        <v>37940</v>
+        <v>38054</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>12986</v>
+        <v>11234</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1168,7 +1168,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.395655632019043</v>
+        <v>4.382145404815674</v>
       </c>
       <c r="C4" s="1">
         <v>1882</v>
@@ -1194,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.9435945153236389</v>
+        <v>0.9406943321228027</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1220,7 +1220,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.780100405216217</v>
+        <v>0.7777027487754822</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1246,7 +1246,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.5418661832809448</v>
+        <v>0.5402007102966309</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1272,7 +1272,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.5325236320495606</v>
+        <v>0.5308868885040283</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.5185098648071289</v>
+        <v>0.5169162154197693</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1324,7 +1324,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.4344271719455719</v>
+        <v>0.433091938495636</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1350,7 +1350,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.4110708832740784</v>
+        <v>0.4098074436187744</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1376,7 +1376,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2896181344985962</v>
+        <v>0.2887279689311981</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1402,7 +1402,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.2569192945957184</v>
+        <v>0.256129652261734</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1428,7 +1428,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.2335630059242249</v>
+        <v>0.2328451275825501</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1454,7 +1454,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1448090672492981</v>
+        <v>0.1443639844655991</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1480,7 +1480,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.1167815029621124</v>
+        <v>0.116422563791275</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1506,7 +1506,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.1167815029621124</v>
+        <v>0.116422563791275</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1532,7 +1532,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.1121102422475815</v>
+        <v>0.111765667796135</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1558,7 +1558,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.0934251993894577</v>
+        <v>0.09313805401325226</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1584,7 +1584,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.08408267796039581</v>
+        <v>0.08382424712181091</v>
       </c>
       <c r="C20" s="1">
         <v>36</v>
@@ -1610,7 +1610,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.08408267796039581</v>
+        <v>0.08382424712181091</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1636,7 +1636,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.07941142469644547</v>
+        <v>0.07916734367609024</v>
       </c>
       <c r="C22" s="1">
         <v>34</v>
@@ -1662,7 +1662,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.07474016398191452</v>
+        <v>0.07451044023036957</v>
       </c>
       <c r="C23" s="1">
         <v>32</v>
@@ -1688,7 +1688,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.07006890326738358</v>
+        <v>0.0698535367846489</v>
       </c>
       <c r="C24" s="1">
         <v>30</v>
@@ -1714,7 +1714,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.07006890326738358</v>
+        <v>0.0698535367846489</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1740,7 +1740,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06539764255285263</v>
+        <v>0.06519664078950882</v>
       </c>
       <c r="C26" s="1">
         <v>28</v>
@@ -1766,7 +1766,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.06539764255285263</v>
+        <v>0.06519664078950882</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1792,7 +1792,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.06539764255285263</v>
+        <v>0.06519664078950882</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1818,7 +1818,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.06539764255285263</v>
+        <v>0.06519664078950882</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1844,7 +1844,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.06072638183832169</v>
+        <v>0.06053973361849785</v>
       </c>
       <c r="C30" s="1">
         <v>26</v>
@@ -1870,7 +1870,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.04204133898019791</v>
+        <v>0.04191212356090546</v>
       </c>
       <c r="C31" s="1">
         <v>18</v>
@@ -1896,7 +1896,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02335629984736443</v>
+        <v>0.02328451350331307</v>
       </c>
       <c r="C32" s="1">
         <v>10</v>
@@ -1922,7 +1922,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01868504099547863</v>
+        <v>0.01862761005759239</v>
       </c>
       <c r="C33" s="1">
         <v>8</v>
@@ -1948,7 +1948,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01868504099547863</v>
+        <v>0.01862761005759239</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1974,7 +1974,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.009342520497739315</v>
+        <v>0.009313805028796196</v>
       </c>
       <c r="C35" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
test pc handle ok
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-8b0af1.o</t>
+    <t>lto-llvm-873e05.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -240,7 +240,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-8b0af1.o</c:v>
+                  <c:v>lto-llvm-873e05.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -335,7 +335,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-8b0af1.o</c:v>
+                  <c:v>lto-llvm-873e05.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>

</xml_diff>

<commit_message>
change set wind to 60
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-873e05.o</t>
+    <t>lto-llvm-b68ff6.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -240,7 +240,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-873e05.o</c:v>
+                  <c:v>lto-llvm-b68ff6.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -335,7 +335,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-873e05.o</c:v>
+                  <c:v>lto-llvm-b68ff6.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -446,103 +446,103 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>89.21461486816406</c:v>
+                  <c:v>89.21662139892578</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.382145404815674</c:v>
+                  <c:v>4.381329536437988</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.9406943321228027</c:v>
+                  <c:v>0.9405191540718079</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.7777027487754822</c:v>
+                  <c:v>0.777557909488678</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.5402007102966309</c:v>
+                  <c:v>0.54010009765625</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.5308868885040283</c:v>
+                  <c:v>0.530788004398346</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.5169162154197693</c:v>
+                  <c:v>0.516819953918457</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.433091938495636</c:v>
+                  <c:v>0.4330112934112549</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4098074436187744</c:v>
+                  <c:v>0.4097311198711395</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2887279689311981</c:v>
+                  <c:v>0.2886742055416107</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.256129652261734</c:v>
+                  <c:v>0.2560819387435913</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2328451275825501</c:v>
+                  <c:v>0.232801765203476</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1443639844655991</c:v>
+                  <c:v>0.1443371027708054</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.116422563791275</c:v>
+                  <c:v>0.116400882601738</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.116422563791275</c:v>
+                  <c:v>0.116400882601738</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.111765667796135</c:v>
+                  <c:v>0.1117448508739471</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.09313805401325226</c:v>
+                  <c:v>0.09312070906162262</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.08382424712181091</c:v>
+                  <c:v>0.08380863815546036</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.08382424712181091</c:v>
+                  <c:v>0.08380863815546036</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.07916734367609024</c:v>
+                  <c:v>0.07915259897708893</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.07451044023036957</c:v>
+                  <c:v>0.0744965672492981</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.0698535367846489</c:v>
+                  <c:v>0.06984052807092667</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.0698535367846489</c:v>
+                  <c:v>0.06984052807092667</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06519664078950882</c:v>
+                  <c:v>0.06518449634313583</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.06519664078950882</c:v>
+                  <c:v>0.06518449634313583</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.06519664078950882</c:v>
+                  <c:v>0.06518449634313583</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.06519664078950882</c:v>
+                  <c:v>0.06518449634313583</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.06053973361849785</c:v>
+                  <c:v>0.0605284608900547</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.04191212356090546</c:v>
+                  <c:v>0.04190431907773018</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02328451350331307</c:v>
+                  <c:v>0.02328017726540566</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01862761005759239</c:v>
+                  <c:v>0.01862414181232452</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01862761005759239</c:v>
+                  <c:v>0.01862414181232452</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.009313805028796196</c:v>
+                  <c:v>0.009312070906162262</c:v>
                 </c:pt>
                 <c:pt idx="33">
                   <c:v>0</c:v>
@@ -1015,10 +1015,10 @@
         <v>11389</v>
       </c>
       <c r="D3" s="1">
-        <v>38315</v>
+        <v>38323</v>
       </c>
       <c r="E3" s="1">
-        <v>38054</v>
+        <v>38062</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1142,16 +1142,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.21461486816406</v>
+        <v>89.21662139892578</v>
       </c>
       <c r="C3" s="1">
-        <v>38315</v>
+        <v>38323</v>
       </c>
       <c r="D3" s="1">
         <v>11389</v>
       </c>
       <c r="E3" s="1">
-        <v>38054</v>
+        <v>38062</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1168,7 +1168,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.382145404815674</v>
+        <v>4.381329536437988</v>
       </c>
       <c r="C4" s="1">
         <v>1882</v>
@@ -1194,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.9406943321228027</v>
+        <v>0.9405191540718079</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1220,7 +1220,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.7777027487754822</v>
+        <v>0.777557909488678</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1246,7 +1246,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.5402007102966309</v>
+        <v>0.54010009765625</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1272,7 +1272,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.5308868885040283</v>
+        <v>0.530788004398346</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.5169162154197693</v>
+        <v>0.516819953918457</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1324,7 +1324,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.433091938495636</v>
+        <v>0.4330112934112549</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1350,7 +1350,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.4098074436187744</v>
+        <v>0.4097311198711395</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1376,7 +1376,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2887279689311981</v>
+        <v>0.2886742055416107</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1402,7 +1402,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.256129652261734</v>
+        <v>0.2560819387435913</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1428,7 +1428,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.2328451275825501</v>
+        <v>0.232801765203476</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1454,7 +1454,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1443639844655991</v>
+        <v>0.1443371027708054</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1480,7 +1480,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.116422563791275</v>
+        <v>0.116400882601738</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1506,7 +1506,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.116422563791275</v>
+        <v>0.116400882601738</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1532,7 +1532,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.111765667796135</v>
+        <v>0.1117448508739471</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1558,7 +1558,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.09313805401325226</v>
+        <v>0.09312070906162262</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1584,7 +1584,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.08382424712181091</v>
+        <v>0.08380863815546036</v>
       </c>
       <c r="C20" s="1">
         <v>36</v>
@@ -1610,7 +1610,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.08382424712181091</v>
+        <v>0.08380863815546036</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1636,7 +1636,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.07916734367609024</v>
+        <v>0.07915259897708893</v>
       </c>
       <c r="C22" s="1">
         <v>34</v>
@@ -1662,7 +1662,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.07451044023036957</v>
+        <v>0.0744965672492981</v>
       </c>
       <c r="C23" s="1">
         <v>32</v>
@@ -1688,7 +1688,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.0698535367846489</v>
+        <v>0.06984052807092667</v>
       </c>
       <c r="C24" s="1">
         <v>30</v>
@@ -1714,7 +1714,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.0698535367846489</v>
+        <v>0.06984052807092667</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1740,7 +1740,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06519664078950882</v>
+        <v>0.06518449634313583</v>
       </c>
       <c r="C26" s="1">
         <v>28</v>
@@ -1766,7 +1766,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.06519664078950882</v>
+        <v>0.06518449634313583</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1792,7 +1792,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.06519664078950882</v>
+        <v>0.06518449634313583</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1818,7 +1818,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.06519664078950882</v>
+        <v>0.06518449634313583</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1844,7 +1844,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.06053973361849785</v>
+        <v>0.0605284608900547</v>
       </c>
       <c r="C30" s="1">
         <v>26</v>
@@ -1870,7 +1870,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.04191212356090546</v>
+        <v>0.04190431907773018</v>
       </c>
       <c r="C31" s="1">
         <v>18</v>
@@ -1896,7 +1896,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02328451350331307</v>
+        <v>0.02328017726540566</v>
       </c>
       <c r="C32" s="1">
         <v>10</v>
@@ -1922,7 +1922,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01862761005759239</v>
+        <v>0.01862414181232452</v>
       </c>
       <c r="C33" s="1">
         <v>8</v>
@@ -1948,7 +1948,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01862761005759239</v>
+        <v>0.01862414181232452</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1974,7 +1974,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.009313805028796196</v>
+        <v>0.009312070906162262</v>
       </c>
       <c r="C35" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
fix channel switch error
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-b68ff6.o</t>
+    <t>lto-llvm-6753d7.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -240,7 +240,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-b68ff6.o</c:v>
+                  <c:v>lto-llvm-6753d7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -335,7 +335,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-b68ff6.o</c:v>
+                  <c:v>lto-llvm-6753d7.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -446,103 +446,103 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>89.21662139892578</c:v>
+                  <c:v>89.31068420410156</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.381329536437988</c:v>
+                  <c:v>4.34311056137085</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.9405191540718079</c:v>
+                  <c:v>0.9323148727416992</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.777557909488678</c:v>
+                  <c:v>0.7707751393318176</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.54010009765625</c:v>
+                  <c:v>0.535388708114624</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.530788004398346</c:v>
+                  <c:v>0.5261579155921936</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.516819953918457</c:v>
+                  <c:v>0.5123116374015808</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4330112934112549</c:v>
+                  <c:v>0.4292340576648712</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4097311198711395</c:v>
+                  <c:v>0.4061569571495056</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2886742055416107</c:v>
+                  <c:v>0.2861560583114624</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.2560819387435913</c:v>
+                  <c:v>0.2538481056690216</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.232801765203476</c:v>
+                  <c:v>0.230771005153656</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1443371027708054</c:v>
+                  <c:v>0.1430780291557312</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.116400882601738</c:v>
+                  <c:v>0.115385502576828</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.116400882601738</c:v>
+                  <c:v>0.115385502576828</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1117448508739471</c:v>
+                  <c:v>0.110770083963871</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.09312070906162262</c:v>
+                  <c:v>0.0923084020614624</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.08380863815546036</c:v>
+                  <c:v>0.0830775648355484</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.08380863815546036</c:v>
+                  <c:v>0.0830775648355484</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.07915259897708893</c:v>
+                  <c:v>0.0784621387720108</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.0744965672492981</c:v>
+                  <c:v>0.0738467201590538</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.06984052807092667</c:v>
+                  <c:v>0.0692313015460968</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.06984052807092667</c:v>
+                  <c:v>0.0692313015460968</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06518449634313583</c:v>
+                  <c:v>0.0646158829331398</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.06518449634313583</c:v>
+                  <c:v>0.0646158829331398</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.06518449634313583</c:v>
+                  <c:v>0.0646158829331398</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.06518449634313583</c:v>
+                  <c:v>0.0646158829331398</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.0605284608900547</c:v>
+                  <c:v>0.0600004605948925</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.04190431907773018</c:v>
+                  <c:v>0.0415387824177742</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02328017726540566</c:v>
+                  <c:v>0.0230771005153656</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01862414181232452</c:v>
+                  <c:v>0.01846168003976345</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01862414181232452</c:v>
+                  <c:v>0.01846168003976345</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.009312070906162262</c:v>
+                  <c:v>0.009230840019881725</c:v>
                 </c:pt>
                 <c:pt idx="33">
                   <c:v>0</c:v>
@@ -1015,10 +1015,10 @@
         <v>11389</v>
       </c>
       <c r="D3" s="1">
-        <v>38323</v>
+        <v>38701</v>
       </c>
       <c r="E3" s="1">
-        <v>38062</v>
+        <v>38440</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1142,16 +1142,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.21662139892578</v>
+        <v>89.31068420410156</v>
       </c>
       <c r="C3" s="1">
-        <v>38323</v>
+        <v>38701</v>
       </c>
       <c r="D3" s="1">
         <v>11389</v>
       </c>
       <c r="E3" s="1">
-        <v>38062</v>
+        <v>38440</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1168,7 +1168,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.381329536437988</v>
+        <v>4.34311056137085</v>
       </c>
       <c r="C4" s="1">
         <v>1882</v>
@@ -1194,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.9405191540718079</v>
+        <v>0.9323148727416992</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1220,7 +1220,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.777557909488678</v>
+        <v>0.7707751393318176</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1246,7 +1246,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.54010009765625</v>
+        <v>0.535388708114624</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1272,7 +1272,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.530788004398346</v>
+        <v>0.5261579155921936</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.516819953918457</v>
+        <v>0.5123116374015808</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1324,7 +1324,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.4330112934112549</v>
+        <v>0.4292340576648712</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1350,7 +1350,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.4097311198711395</v>
+        <v>0.4061569571495056</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1376,7 +1376,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2886742055416107</v>
+        <v>0.2861560583114624</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1402,7 +1402,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.2560819387435913</v>
+        <v>0.2538481056690216</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1428,7 +1428,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.232801765203476</v>
+        <v>0.230771005153656</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1454,7 +1454,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1443371027708054</v>
+        <v>0.1430780291557312</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1480,7 +1480,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.116400882601738</v>
+        <v>0.115385502576828</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1506,7 +1506,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.116400882601738</v>
+        <v>0.115385502576828</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1532,7 +1532,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.1117448508739471</v>
+        <v>0.110770083963871</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1558,7 +1558,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.09312070906162262</v>
+        <v>0.0923084020614624</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1584,7 +1584,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.08380863815546036</v>
+        <v>0.0830775648355484</v>
       </c>
       <c r="C20" s="1">
         <v>36</v>
@@ -1610,7 +1610,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.08380863815546036</v>
+        <v>0.0830775648355484</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1636,7 +1636,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.07915259897708893</v>
+        <v>0.0784621387720108</v>
       </c>
       <c r="C22" s="1">
         <v>34</v>
@@ -1662,7 +1662,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.0744965672492981</v>
+        <v>0.0738467201590538</v>
       </c>
       <c r="C23" s="1">
         <v>32</v>
@@ -1688,7 +1688,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.06984052807092667</v>
+        <v>0.0692313015460968</v>
       </c>
       <c r="C24" s="1">
         <v>30</v>
@@ -1714,7 +1714,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.06984052807092667</v>
+        <v>0.0692313015460968</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1740,7 +1740,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06518449634313583</v>
+        <v>0.0646158829331398</v>
       </c>
       <c r="C26" s="1">
         <v>28</v>
@@ -1766,7 +1766,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.06518449634313583</v>
+        <v>0.0646158829331398</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1792,7 +1792,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.06518449634313583</v>
+        <v>0.0646158829331398</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1818,7 +1818,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.06518449634313583</v>
+        <v>0.0646158829331398</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1844,7 +1844,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.0605284608900547</v>
+        <v>0.0600004605948925</v>
       </c>
       <c r="C30" s="1">
         <v>26</v>
@@ -1870,7 +1870,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.04190431907773018</v>
+        <v>0.0415387824177742</v>
       </c>
       <c r="C31" s="1">
         <v>18</v>
@@ -1896,7 +1896,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02328017726540566</v>
+        <v>0.0230771005153656</v>
       </c>
       <c r="C32" s="1">
         <v>10</v>
@@ -1922,7 +1922,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01862414181232452</v>
+        <v>0.01846168003976345</v>
       </c>
       <c r="C33" s="1">
         <v>8</v>
@@ -1948,7 +1948,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01862414181232452</v>
+        <v>0.01846168003976345</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1974,7 +1974,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.009312070906162262</v>
+        <v>0.009230840019881725</v>
       </c>
       <c r="C35" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
fix voice control error
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-6753d7.o</t>
+    <t>lto-llvm-4c9ad1.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -240,7 +240,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-6753d7.o</c:v>
+                  <c:v>lto-llvm-4c9ad1.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -335,7 +335,7 @@
               <c:strCache>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-6753d7.o</c:v>
+                  <c:v>lto-llvm-4c9ad1.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -446,103 +446,103 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="34"/>
                 <c:pt idx="0">
-                  <c:v>89.31068420410156</c:v>
+                  <c:v>89.32398986816406</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.34311056137085</c:v>
+                  <c:v>4.337704658508301</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.9323148727416992</c:v>
+                  <c:v>0.9311544895172119</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.7707751393318176</c:v>
+                  <c:v>0.7698158621788025</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.535388708114624</c:v>
+                  <c:v>0.5347223877906799</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.5261579155921936</c:v>
+                  <c:v>0.5255030393600464</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.5123116374015808</c:v>
+                  <c:v>0.5116739869117737</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4292340576648712</c:v>
+                  <c:v>0.4286998510360718</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4061569571495056</c:v>
+                  <c:v>0.4056514501571655</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2861560583114624</c:v>
+                  <c:v>0.2857998907566071</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.2538481056690216</c:v>
+                  <c:v>0.2535321712493897</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.230771005153656</c:v>
+                  <c:v>0.2304837852716446</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1430780291557312</c:v>
+                  <c:v>0.1428999453783035</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.115385502576828</c:v>
+                  <c:v>0.1152418926358223</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.115385502576828</c:v>
+                  <c:v>0.1152418926358223</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.110770083963871</c:v>
+                  <c:v>0.1106322184205055</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.0923084020614624</c:v>
+                  <c:v>0.09219351410865784</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.0830775648355484</c:v>
+                  <c:v>0.08297416567802429</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.0830775648355484</c:v>
+                  <c:v>0.08297416567802429</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.0784621387720108</c:v>
+                  <c:v>0.07836448401212692</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.0738467201590538</c:v>
+                  <c:v>0.07375480979681015</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.0692313015460968</c:v>
+                  <c:v>0.06914513558149338</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.0692313015460968</c:v>
+                  <c:v>0.06914513558149338</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.0646158829331398</c:v>
+                  <c:v>0.06453546136617661</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.0646158829331398</c:v>
+                  <c:v>0.06453546136617661</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.0646158829331398</c:v>
+                  <c:v>0.06453546136617661</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.0646158829331398</c:v>
+                  <c:v>0.06453546136617661</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.0600004605948925</c:v>
+                  <c:v>0.05992578342556953</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.0415387824177742</c:v>
+                  <c:v>0.04148708283901215</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.0230771005153656</c:v>
+                  <c:v>0.02304837852716446</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01846168003976345</c:v>
+                  <c:v>0.01843870244920254</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01846168003976345</c:v>
+                  <c:v>0.01843870244920254</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.009230840019881725</c:v>
+                  <c:v>0.009219351224601269</c:v>
                 </c:pt>
                 <c:pt idx="33">
                   <c:v>0</c:v>
@@ -1015,10 +1015,10 @@
         <v>11389</v>
       </c>
       <c r="D3" s="1">
-        <v>38701</v>
+        <v>38755</v>
       </c>
       <c r="E3" s="1">
-        <v>38440</v>
+        <v>38494</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1142,16 +1142,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.31068420410156</v>
+        <v>89.32398986816406</v>
       </c>
       <c r="C3" s="1">
-        <v>38701</v>
+        <v>38755</v>
       </c>
       <c r="D3" s="1">
         <v>11389</v>
       </c>
       <c r="E3" s="1">
-        <v>38440</v>
+        <v>38494</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1168,7 +1168,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.34311056137085</v>
+        <v>4.337704658508301</v>
       </c>
       <c r="C4" s="1">
         <v>1882</v>
@@ -1194,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.9323148727416992</v>
+        <v>0.9311544895172119</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1220,7 +1220,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.7707751393318176</v>
+        <v>0.7698158621788025</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1246,7 +1246,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.535388708114624</v>
+        <v>0.5347223877906799</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1272,7 +1272,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.5261579155921936</v>
+        <v>0.5255030393600464</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.5123116374015808</v>
+        <v>0.5116739869117737</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1324,7 +1324,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.4292340576648712</v>
+        <v>0.4286998510360718</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1350,7 +1350,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.4061569571495056</v>
+        <v>0.4056514501571655</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1376,7 +1376,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2861560583114624</v>
+        <v>0.2857998907566071</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1402,7 +1402,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.2538481056690216</v>
+        <v>0.2535321712493897</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1428,7 +1428,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.230771005153656</v>
+        <v>0.2304837852716446</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1454,7 +1454,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1430780291557312</v>
+        <v>0.1428999453783035</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1480,7 +1480,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.115385502576828</v>
+        <v>0.1152418926358223</v>
       </c>
       <c r="C16" s="1">
         <v>50</v>
@@ -1506,7 +1506,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.115385502576828</v>
+        <v>0.1152418926358223</v>
       </c>
       <c r="C17" s="1">
         <v>50</v>
@@ -1532,7 +1532,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.110770083963871</v>
+        <v>0.1106322184205055</v>
       </c>
       <c r="C18" s="1">
         <v>48</v>
@@ -1558,7 +1558,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.0923084020614624</v>
+        <v>0.09219351410865784</v>
       </c>
       <c r="C19" s="1">
         <v>40</v>
@@ -1584,7 +1584,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.0830775648355484</v>
+        <v>0.08297416567802429</v>
       </c>
       <c r="C20" s="1">
         <v>36</v>
@@ -1610,7 +1610,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.0830775648355484</v>
+        <v>0.08297416567802429</v>
       </c>
       <c r="C21" s="1">
         <v>36</v>
@@ -1636,7 +1636,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.0784621387720108</v>
+        <v>0.07836448401212692</v>
       </c>
       <c r="C22" s="1">
         <v>34</v>
@@ -1662,7 +1662,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.0738467201590538</v>
+        <v>0.07375480979681015</v>
       </c>
       <c r="C23" s="1">
         <v>32</v>
@@ -1688,7 +1688,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.0692313015460968</v>
+        <v>0.06914513558149338</v>
       </c>
       <c r="C24" s="1">
         <v>30</v>
@@ -1714,7 +1714,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.0692313015460968</v>
+        <v>0.06914513558149338</v>
       </c>
       <c r="C25" s="1">
         <v>30</v>
@@ -1740,7 +1740,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.0646158829331398</v>
+        <v>0.06453546136617661</v>
       </c>
       <c r="C26" s="1">
         <v>28</v>
@@ -1766,7 +1766,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.0646158829331398</v>
+        <v>0.06453546136617661</v>
       </c>
       <c r="C27" s="1">
         <v>28</v>
@@ -1792,7 +1792,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.0646158829331398</v>
+        <v>0.06453546136617661</v>
       </c>
       <c r="C28" s="1">
         <v>28</v>
@@ -1818,7 +1818,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.0646158829331398</v>
+        <v>0.06453546136617661</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1844,7 +1844,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.0600004605948925</v>
+        <v>0.05992578342556953</v>
       </c>
       <c r="C30" s="1">
         <v>26</v>
@@ -1870,7 +1870,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.0415387824177742</v>
+        <v>0.04148708283901215</v>
       </c>
       <c r="C31" s="1">
         <v>18</v>
@@ -1896,7 +1896,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.0230771005153656</v>
+        <v>0.02304837852716446</v>
       </c>
       <c r="C32" s="1">
         <v>10</v>
@@ -1922,7 +1922,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01846168003976345</v>
+        <v>0.01843870244920254</v>
       </c>
       <c r="C33" s="1">
         <v>8</v>
@@ -1948,7 +1948,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01846168003976345</v>
+        <v>0.01843870244920254</v>
       </c>
       <c r="C34" s="1">
         <v>8</v>
@@ -1974,7 +1974,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.009230840019881725</v>
+        <v>0.009219351224601269</v>
       </c>
       <c r="C35" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
change output value,software V1.4.2
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
   <si>
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-4c9ad1.o</t>
+    <t>lto-llvm-c21010.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -59,6 +59,12 @@
     <t>dfixi.o</t>
   </si>
   <si>
+    <t>d2f.o</t>
+  </si>
+  <si>
+    <t>dcmpgt.o</t>
+  </si>
+  <si>
     <t>ffixi.o</t>
   </si>
   <si>
@@ -69,6 +75,9 @@
   </si>
   <si>
     <t>ffixui.o</t>
+  </si>
+  <si>
+    <t>f2d.o</t>
   </si>
   <si>
     <t>memseta.o</t>
@@ -236,16 +245,16 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>ram_percent!$A$3:$A$36</c:f>
+              <c:f>ram_percent!$A$3:$A$39</c:f>
               <c:strCache>
-                <c:ptCount val="34"/>
+                <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-4c9ad1.o</c:v>
+                  <c:v>lto-llvm-c21010.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
                 </c:pt>
-                <c:pt idx="33">
+                <c:pt idx="36">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -253,17 +262,17 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>ram_percent!$B$3:$B$36</c:f>
+              <c:f>ram_percent!$B$3:$B$39</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="34"/>
+                <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>91.75058746337891</c:v>
+                  <c:v>91.73993682861328</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.249416351318359</c:v>
-                </c:pt>
-                <c:pt idx="33">
+                  <c:v>8.260063171386719</c:v>
+                </c:pt>
+                <c:pt idx="36">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -331,11 +340,11 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>flash_percent!$A$3:$A$36</c:f>
+              <c:f>flash_percent!$A$3:$A$39</c:f>
               <c:strCache>
-                <c:ptCount val="34"/>
+                <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-4c9ad1.o</c:v>
+                  <c:v>lto-llvm-c21010.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -374,66 +383,75 @@
                   <c:v>dfixi.o</c:v>
                 </c:pt>
                 <c:pt idx="13">
+                  <c:v>d2f.o</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>dcmpgt.o</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>ffixi.o</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="16">
                   <c:v>dfixui.o</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="17">
                   <c:v>init.o</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="18">
                   <c:v>ffixui.o</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="19">
+                  <c:v>f2d.o</c:v>
+                </c:pt>
+                <c:pt idx="20">
                   <c:v>memseta.o</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="21">
                   <c:v>llsshr.o</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="22">
                   <c:v>dflti.o</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="23">
                   <c:v>llushr.o</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="24">
                   <c:v>llshl.o</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="25">
                   <c:v>handlers.o</c:v>
                 </c:pt>
-                <c:pt idx="23">
+                <c:pt idx="26">
                   <c:v>fcmplt.o</c:v>
                 </c:pt>
-                <c:pt idx="24">
+                <c:pt idx="27">
                   <c:v>fcmple.o</c:v>
                 </c:pt>
-                <c:pt idx="25">
+                <c:pt idx="28">
                   <c:v>fcmpgt.o</c:v>
                 </c:pt>
-                <c:pt idx="26">
+                <c:pt idx="29">
                   <c:v>fcmpge.o</c:v>
                 </c:pt>
-                <c:pt idx="27">
+                <c:pt idx="30">
                   <c:v>dfltui.o</c:v>
                 </c:pt>
-                <c:pt idx="28">
+                <c:pt idx="31">
                   <c:v>fflti.o</c:v>
                 </c:pt>
-                <c:pt idx="29">
+                <c:pt idx="32">
                   <c:v>ffltui.o</c:v>
                 </c:pt>
-                <c:pt idx="30">
+                <c:pt idx="33">
                   <c:v>entry9a.o</c:v>
                 </c:pt>
-                <c:pt idx="31">
+                <c:pt idx="34">
                   <c:v>entry2.o</c:v>
                 </c:pt>
-                <c:pt idx="32">
+                <c:pt idx="35">
                   <c:v>entry5.o</c:v>
                 </c:pt>
-                <c:pt idx="33">
+                <c:pt idx="36">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -441,110 +459,119 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>flash_percent!$B$3:$B$36</c:f>
+              <c:f>flash_percent!$B$3:$B$39</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="34"/>
+                <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>89.32398986816406</c:v>
+                  <c:v>88.81499481201172</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.337704658508301</c:v>
+                  <c:v>4.607458114624023</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.9311544895172119</c:v>
+                  <c:v>0.9169522523880005</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.7698158621788025</c:v>
+                  <c:v>0.7580744028091431</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.5347223877906799</c:v>
+                  <c:v>0.5265666246414185</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.5255030393600464</c:v>
+                  <c:v>0.5174879431724548</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.5116739869117737</c:v>
+                  <c:v>0.5038698315620422</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4286998510360718</c:v>
+                  <c:v>0.422161191701889</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4056514501571655</c:v>
+                  <c:v>0.3994643688201904</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2857998907566071</c:v>
+                  <c:v>0.281440794467926</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.2535321712493897</c:v>
+                  <c:v>0.2496652156114578</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2304837852716446</c:v>
+                  <c:v>0.226968377828598</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1428999453783035</c:v>
+                  <c:v>0.140720397233963</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.1152418926358223</c:v>
+                  <c:v>0.1271023005247116</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.1152418926358223</c:v>
+                  <c:v>0.1225629299879074</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1106322184205055</c:v>
+                  <c:v>0.113484188914299</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.09219351410865784</c:v>
+                  <c:v>0.113484188914299</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.08297416567802429</c:v>
+                  <c:v>0.1089448258280754</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.08297416567802429</c:v>
+                  <c:v>0.09078735113143921</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.07836448401212692</c:v>
+                  <c:v>0.08624798804521561</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.07375480979681015</c:v>
+                  <c:v>0.08170861750841141</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.06914513558149338</c:v>
+                  <c:v>0.08170861750841141</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.06914513558149338</c:v>
+                  <c:v>0.07716924697160721</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06453546136617661</c:v>
+                  <c:v>0.07262988388538361</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.06453546136617661</c:v>
+                  <c:v>0.06809051334857941</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.06453546136617661</c:v>
+                  <c:v>0.06809051334857941</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.06453546136617661</c:v>
+                  <c:v>0.0635511502623558</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.05992578342556953</c:v>
+                  <c:v>0.0635511502623558</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.04148708283901215</c:v>
+                  <c:v>0.0635511502623558</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.02304837852716446</c:v>
+                  <c:v>0.0635511502623558</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.01843870244920254</c:v>
+                  <c:v>0.05901177972555161</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.01843870244920254</c:v>
+                  <c:v>0.0408543087542057</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.009219351224601269</c:v>
+                  <c:v>0.0226968377828598</c:v>
                 </c:pt>
                 <c:pt idx="33">
+                  <c:v>0.0181574709713459</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.0181574709713459</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.009078735485672951</c:v>
+                </c:pt>
+                <c:pt idx="36">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -649,8 +676,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H36" totalsRowCount="1">
-  <autoFilter ref="A2:H35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H39" totalsRowCount="1">
+  <autoFilter ref="A2:H38"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="ram_percent" totalsRowFunction="sum"/>
@@ -666,8 +693,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H36" totalsRowCount="1">
-  <autoFilter ref="A2:H35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H39" totalsRowCount="1">
+  <autoFilter ref="A2:H38"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="flash_percent" totalsRowFunction="sum"/>
@@ -967,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -980,28 +1007,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1009,16 +1036,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.75058746337891</v>
+        <v>91.73993682861328</v>
       </c>
       <c r="C3" s="1">
-        <v>11389</v>
+        <v>11373</v>
       </c>
       <c r="D3" s="1">
-        <v>38755</v>
+        <v>39131</v>
       </c>
       <c r="E3" s="1">
-        <v>38494</v>
+        <v>38870</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1027,7 +1054,7 @@
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11234</v>
+        <v>11218</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1035,7 +1062,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.249416351318359</v>
+        <v>8.260063171386719</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1056,35 +1083,35 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36">
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
         <f>SUBTOTAL(109,[ram_percent])</f>
         <v>0</v>
       </c>
-      <c r="C36">
+      <c r="C39">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="D36">
+      <c r="D39">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="E36">
+      <c r="E39">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F36">
+      <c r="F39">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G36">
+      <c r="G39">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H36">
+      <c r="H39">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>
@@ -1100,7 +1127,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1113,28 +1140,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" t="s">
-        <v>40</v>
-      </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1142,16 +1169,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.32398986816406</v>
+        <v>88.81499481201172</v>
       </c>
       <c r="C3" s="1">
-        <v>38755</v>
+        <v>39131</v>
       </c>
       <c r="D3" s="1">
-        <v>11389</v>
+        <v>11373</v>
       </c>
       <c r="E3" s="1">
-        <v>38494</v>
+        <v>38870</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
@@ -1160,7 +1187,7 @@
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11234</v>
+        <v>11218</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1168,16 +1195,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.337704658508301</v>
+        <v>4.607458114624023</v>
       </c>
       <c r="C4" s="1">
-        <v>1882</v>
+        <v>2030</v>
       </c>
       <c r="D4" s="1">
         <v>0</v>
       </c>
       <c r="E4" s="1">
-        <v>1882</v>
+        <v>2030</v>
       </c>
       <c r="F4" s="1">
         <v>0</v>
@@ -1194,7 +1221,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.9311544895172119</v>
+        <v>0.9169522523880005</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1220,7 +1247,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.7698158621788025</v>
+        <v>0.7580744028091431</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1246,7 +1273,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.5347223877906799</v>
+        <v>0.5265666246414185</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1272,7 +1299,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.5255030393600464</v>
+        <v>0.5174879431724548</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1298,7 +1325,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.5116739869117737</v>
+        <v>0.5038698315620422</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1324,7 +1351,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.4286998510360718</v>
+        <v>0.422161191701889</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1350,7 +1377,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.4056514501571655</v>
+        <v>0.3994643688201904</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1376,7 +1403,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2857998907566071</v>
+        <v>0.281440794467926</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1402,7 +1429,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.2535321712493897</v>
+        <v>0.2496652156114578</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1428,7 +1455,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.2304837852716446</v>
+        <v>0.226968377828598</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1454,7 +1481,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1428999453783035</v>
+        <v>0.140720397233963</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1480,16 +1507,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.1152418926358223</v>
+        <v>0.1271023005247116</v>
       </c>
       <c r="C16" s="1">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -1506,16 +1533,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.1152418926358223</v>
+        <v>0.1225629299879074</v>
       </c>
       <c r="C17" s="1">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D17" s="1">
         <v>0</v>
       </c>
       <c r="E17" s="1">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F17" s="1">
         <v>0</v>
@@ -1532,16 +1559,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.1106322184205055</v>
+        <v>0.113484188914299</v>
       </c>
       <c r="C18" s="1">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -1558,16 +1585,16 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.09219351410865784</v>
+        <v>0.113484188914299</v>
       </c>
       <c r="C19" s="1">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D19" s="1">
         <v>0</v>
       </c>
       <c r="E19" s="1">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
@@ -1584,16 +1611,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.08297416567802429</v>
+        <v>0.1089448258280754</v>
       </c>
       <c r="C20" s="1">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
@@ -1610,16 +1637,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.08297416567802429</v>
+        <v>0.09078735113143921</v>
       </c>
       <c r="C21" s="1">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D21" s="1">
         <v>0</v>
       </c>
       <c r="E21" s="1">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F21" s="1">
         <v>0</v>
@@ -1636,16 +1663,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.07836448401212692</v>
+        <v>0.08624798804521561</v>
       </c>
       <c r="C22" s="1">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D22" s="1">
         <v>0</v>
       </c>
       <c r="E22" s="1">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F22" s="1">
         <v>0</v>
@@ -1662,16 +1689,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.07375480979681015</v>
+        <v>0.08170861750841141</v>
       </c>
       <c r="C23" s="1">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D23" s="1">
         <v>0</v>
       </c>
       <c r="E23" s="1">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F23" s="1">
         <v>0</v>
@@ -1688,16 +1715,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.06914513558149338</v>
+        <v>0.08170861750841141</v>
       </c>
       <c r="C24" s="1">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D24" s="1">
         <v>0</v>
       </c>
       <c r="E24" s="1">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F24" s="1">
         <v>0</v>
@@ -1714,16 +1741,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.06914513558149338</v>
+        <v>0.07716924697160721</v>
       </c>
       <c r="C25" s="1">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -1740,16 +1767,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06453546136617661</v>
+        <v>0.07262988388538361</v>
       </c>
       <c r="C26" s="1">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D26" s="1">
         <v>0</v>
       </c>
       <c r="E26" s="1">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F26" s="1">
         <v>0</v>
@@ -1766,16 +1793,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.06453546136617661</v>
+        <v>0.06809051334857941</v>
       </c>
       <c r="C27" s="1">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D27" s="1">
         <v>0</v>
       </c>
       <c r="E27" s="1">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F27" s="1">
         <v>0</v>
@@ -1792,16 +1819,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.06453546136617661</v>
+        <v>0.06809051334857941</v>
       </c>
       <c r="C28" s="1">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D28" s="1">
         <v>0</v>
       </c>
       <c r="E28" s="1">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F28" s="1">
         <v>0</v>
@@ -1818,7 +1845,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.06453546136617661</v>
+        <v>0.0635511502623558</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1844,16 +1871,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.05992578342556953</v>
+        <v>0.0635511502623558</v>
       </c>
       <c r="C30" s="1">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D30" s="1">
         <v>0</v>
       </c>
       <c r="E30" s="1">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F30" s="1">
         <v>0</v>
@@ -1870,16 +1897,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.04148708283901215</v>
+        <v>0.0635511502623558</v>
       </c>
       <c r="C31" s="1">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D31" s="1">
         <v>0</v>
       </c>
       <c r="E31" s="1">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F31" s="1">
         <v>0</v>
@@ -1896,16 +1923,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.02304837852716446</v>
+        <v>0.0635511502623558</v>
       </c>
       <c r="C32" s="1">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D32" s="1">
         <v>0</v>
       </c>
       <c r="E32" s="1">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F32" s="1">
         <v>0</v>
@@ -1922,16 +1949,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.01843870244920254</v>
+        <v>0.05901177972555161</v>
       </c>
       <c r="C33" s="1">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D33" s="1">
         <v>0</v>
       </c>
       <c r="E33" s="1">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
@@ -1948,16 +1975,16 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.01843870244920254</v>
+        <v>0.0408543087542057</v>
       </c>
       <c r="C34" s="1">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D34" s="1">
         <v>0</v>
       </c>
       <c r="E34" s="1">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F34" s="1">
         <v>0</v>
@@ -1974,56 +2001,134 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.009219351224601269</v>
+        <v>0.0226968377828598</v>
       </c>
       <c r="C35" s="1">
+        <v>10</v>
+      </c>
+      <c r="D35" s="1">
+        <v>0</v>
+      </c>
+      <c r="E35" s="1">
+        <v>10</v>
+      </c>
+      <c r="F35" s="1">
+        <v>0</v>
+      </c>
+      <c r="G35" s="1">
+        <v>0</v>
+      </c>
+      <c r="H35" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" s="2">
+        <v>0.0181574709713459</v>
+      </c>
+      <c r="C36" s="1">
+        <v>8</v>
+      </c>
+      <c r="D36" s="1">
+        <v>0</v>
+      </c>
+      <c r="E36" s="1">
+        <v>8</v>
+      </c>
+      <c r="F36" s="1">
+        <v>0</v>
+      </c>
+      <c r="G36" s="1">
+        <v>0</v>
+      </c>
+      <c r="H36" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" s="2">
+        <v>0.0181574709713459</v>
+      </c>
+      <c r="C37" s="1">
+        <v>8</v>
+      </c>
+      <c r="D37" s="1">
+        <v>0</v>
+      </c>
+      <c r="E37" s="1">
+        <v>8</v>
+      </c>
+      <c r="F37" s="1">
+        <v>0</v>
+      </c>
+      <c r="G37" s="1">
+        <v>0</v>
+      </c>
+      <c r="H37" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="2">
+        <v>0.009078735485672951</v>
+      </c>
+      <c r="C38" s="1">
         <v>4</v>
       </c>
-      <c r="D35" s="1">
-        <v>0</v>
-      </c>
-      <c r="E35" s="1">
+      <c r="D38" s="1">
+        <v>0</v>
+      </c>
+      <c r="E38" s="1">
         <v>4</v>
       </c>
-      <c r="F35" s="1">
-        <v>0</v>
-      </c>
-      <c r="G35" s="1">
-        <v>0</v>
-      </c>
-      <c r="H35" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36">
+      <c r="F38" s="1">
+        <v>0</v>
+      </c>
+      <c r="G38" s="1">
+        <v>0</v>
+      </c>
+      <c r="H38" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
         <f>SUBTOTAL(109,[flash_percent])</f>
         <v>0</v>
       </c>
-      <c r="C36">
+      <c r="C39">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="D36">
+      <c r="D39">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="E36">
+      <c r="E39">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F36">
+      <c r="F39">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G36">
+      <c r="G39">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H36">
+      <c r="H39">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
change setting temp and wind refresh time to slow
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-79bc84.o</t>
+    <t>lto-llvm-2aa6ce.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -249,7 +249,7 @@
               <c:strCache>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-79bc84.o</c:v>
+                  <c:v>lto-llvm-2aa6ce.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -267,10 +267,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>91.75656127929688</c:v>
+                  <c:v>91.75921630859375</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.243438720703125</c:v>
+                  <c:v>8.240785598754883</c:v>
                 </c:pt>
                 <c:pt idx="36">
                   <c:v>0</c:v>
@@ -344,7 +344,7 @@
               <c:strCache>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-79bc84.o</c:v>
+                  <c:v>lto-llvm-2aa6ce.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -464,112 +464,112 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>89.2255859375</c:v>
+                  <c:v>89.24064636230469</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.4383225440979</c:v>
+                  <c:v>4.432120800018311</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8832917809486389</c:v>
+                  <c:v>0.8820575475692749</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.7302461862564087</c:v>
+                  <c:v>0.7292258143424988</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.5072368979454041</c:v>
+                  <c:v>0.5065280795097351</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.4984914064407349</c:v>
+                  <c:v>0.4977948665618897</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.4853731989860535</c:v>
+                  <c:v>0.4846949875354767</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4066640436649323</c:v>
+                  <c:v>0.4060958027839661</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3848003745079041</c:v>
+                  <c:v>0.3842627108097076</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2711093723773956</c:v>
+                  <c:v>0.2707305252552033</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.2405002415180206</c:v>
+                  <c:v>0.240164190530777</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2186365872621536</c:v>
+                  <c:v>0.2183310836553574</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1355546861886978</c:v>
+                  <c:v>0.1353652626276016</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.122436486184597</c:v>
+                  <c:v>0.1222654059529305</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.1180637553334236</c:v>
+                  <c:v>0.1178987845778465</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1093182936310768</c:v>
+                  <c:v>0.1091655418276787</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.1093182936310768</c:v>
+                  <c:v>0.1091655418276787</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.1049455627799034</c:v>
+                  <c:v>0.1047989204525948</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.08745463192462921</c:v>
+                  <c:v>0.08733242750167847</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.08308190107345581</c:v>
+                  <c:v>0.08296580612659454</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.07870917022228241</c:v>
+                  <c:v>0.07859918475151062</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.07870917022228241</c:v>
+                  <c:v>0.07859918475151062</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.07433643937110901</c:v>
+                  <c:v>0.0742325633764267</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06996370851993561</c:v>
+                  <c:v>0.06986594200134277</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.06559097766876221</c:v>
+                  <c:v>0.06549932062625885</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.06559097766876221</c:v>
+                  <c:v>0.06549932062625885</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.06121824309229851</c:v>
+                  <c:v>0.06113270297646523</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.06121824309229851</c:v>
+                  <c:v>0.06113270297646523</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.06121824309229851</c:v>
+                  <c:v>0.06113270297646523</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.06121824309229851</c:v>
+                  <c:v>0.06113270297646523</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.05684551224112511</c:v>
+                  <c:v>0.0567660816013813</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.03935458511114121</c:v>
+                  <c:v>0.03929959237575531</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.0218636579811573</c:v>
+                  <c:v>0.02183310687541962</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.0174909271299839</c:v>
+                  <c:v>0.01746648550033569</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.0174909271299839</c:v>
+                  <c:v>0.01746648550033569</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.008745463564991951</c:v>
+                  <c:v>0.008733242750167847</c:v>
                 </c:pt>
                 <c:pt idx="36">
                   <c:v>0</c:v>
@@ -1036,22 +1036,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.75656127929688</v>
+        <v>91.75921630859375</v>
       </c>
       <c r="C3" s="1">
-        <v>11398</v>
+        <v>11402</v>
       </c>
       <c r="D3" s="1">
-        <v>40810</v>
+        <v>40874</v>
       </c>
       <c r="E3" s="1">
-        <v>40548</v>
+        <v>40608</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H3" s="1">
         <v>11242</v>
@@ -1062,7 +1062,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.243438720703125</v>
+        <v>8.240785598754883</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1169,22 +1169,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.2255859375</v>
+        <v>89.24064636230469</v>
       </c>
       <c r="C3" s="1">
-        <v>40810</v>
+        <v>40874</v>
       </c>
       <c r="D3" s="1">
-        <v>11398</v>
+        <v>11402</v>
       </c>
       <c r="E3" s="1">
-        <v>40548</v>
+        <v>40608</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H3" s="1">
         <v>11242</v>
@@ -1195,7 +1195,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.4383225440979</v>
+        <v>4.432120800018311</v>
       </c>
       <c r="C4" s="1">
         <v>2030</v>
@@ -1221,7 +1221,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.8832917809486389</v>
+        <v>0.8820575475692749</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1247,7 +1247,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.7302461862564087</v>
+        <v>0.7292258143424988</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1273,7 +1273,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.5072368979454041</v>
+        <v>0.5065280795097351</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1299,7 +1299,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.4984914064407349</v>
+        <v>0.4977948665618897</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1325,7 +1325,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.4853731989860535</v>
+        <v>0.4846949875354767</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1351,7 +1351,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.4066640436649323</v>
+        <v>0.4060958027839661</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1377,7 +1377,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.3848003745079041</v>
+        <v>0.3842627108097076</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1403,7 +1403,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2711093723773956</v>
+        <v>0.2707305252552033</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1429,7 +1429,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.2405002415180206</v>
+        <v>0.240164190530777</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1455,7 +1455,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.2186365872621536</v>
+        <v>0.2183310836553574</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1481,7 +1481,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1355546861886978</v>
+        <v>0.1353652626276016</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1507,7 +1507,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.122436486184597</v>
+        <v>0.1222654059529305</v>
       </c>
       <c r="C16" s="1">
         <v>56</v>
@@ -1533,7 +1533,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.1180637553334236</v>
+        <v>0.1178987845778465</v>
       </c>
       <c r="C17" s="1">
         <v>54</v>
@@ -1559,7 +1559,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.1093182936310768</v>
+        <v>0.1091655418276787</v>
       </c>
       <c r="C18" s="1">
         <v>50</v>
@@ -1585,7 +1585,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.1093182936310768</v>
+        <v>0.1091655418276787</v>
       </c>
       <c r="C19" s="1">
         <v>50</v>
@@ -1611,7 +1611,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.1049455627799034</v>
+        <v>0.1047989204525948</v>
       </c>
       <c r="C20" s="1">
         <v>48</v>
@@ -1637,7 +1637,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.08745463192462921</v>
+        <v>0.08733242750167847</v>
       </c>
       <c r="C21" s="1">
         <v>40</v>
@@ -1663,7 +1663,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.08308190107345581</v>
+        <v>0.08296580612659454</v>
       </c>
       <c r="C22" s="1">
         <v>38</v>
@@ -1689,7 +1689,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.07870917022228241</v>
+        <v>0.07859918475151062</v>
       </c>
       <c r="C23" s="1">
         <v>36</v>
@@ -1715,7 +1715,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.07870917022228241</v>
+        <v>0.07859918475151062</v>
       </c>
       <c r="C24" s="1">
         <v>36</v>
@@ -1741,7 +1741,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.07433643937110901</v>
+        <v>0.0742325633764267</v>
       </c>
       <c r="C25" s="1">
         <v>34</v>
@@ -1767,7 +1767,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06996370851993561</v>
+        <v>0.06986594200134277</v>
       </c>
       <c r="C26" s="1">
         <v>32</v>
@@ -1793,7 +1793,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.06559097766876221</v>
+        <v>0.06549932062625885</v>
       </c>
       <c r="C27" s="1">
         <v>30</v>
@@ -1819,7 +1819,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.06559097766876221</v>
+        <v>0.06549932062625885</v>
       </c>
       <c r="C28" s="1">
         <v>30</v>
@@ -1845,7 +1845,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.06121824309229851</v>
+        <v>0.06113270297646523</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1871,7 +1871,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.06121824309229851</v>
+        <v>0.06113270297646523</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1897,7 +1897,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.06121824309229851</v>
+        <v>0.06113270297646523</v>
       </c>
       <c r="C31" s="1">
         <v>28</v>
@@ -1923,7 +1923,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.06121824309229851</v>
+        <v>0.06113270297646523</v>
       </c>
       <c r="C32" s="1">
         <v>28</v>
@@ -1949,7 +1949,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.05684551224112511</v>
+        <v>0.0567660816013813</v>
       </c>
       <c r="C33" s="1">
         <v>26</v>
@@ -1975,7 +1975,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.03935458511114121</v>
+        <v>0.03929959237575531</v>
       </c>
       <c r="C34" s="1">
         <v>18</v>
@@ -2001,7 +2001,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.0218636579811573</v>
+        <v>0.02183310687541962</v>
       </c>
       <c r="C35" s="1">
         <v>10</v>
@@ -2027,7 +2027,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.0174909271299839</v>
+        <v>0.01746648550033569</v>
       </c>
       <c r="C36" s="1">
         <v>8</v>
@@ -2053,7 +2053,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="2">
-        <v>0.0174909271299839</v>
+        <v>0.01746648550033569</v>
       </c>
       <c r="C37" s="1">
         <v>8</v>
@@ -2079,7 +2079,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="2">
-        <v>0.008745463564991951</v>
+        <v>0.008733242750167847</v>
       </c>
       <c r="C38" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
fix always setting wind when pick up handle in first software V1.4.3
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-2aa6ce.o</t>
+    <t>lto-llvm-30d3b0.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -249,7 +249,7 @@
               <c:strCache>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-2aa6ce.o</c:v>
+                  <c:v>lto-llvm-30d3b0.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -267,10 +267,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>91.75921630859375</c:v>
+                  <c:v>91.76385498046875</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.240785598754883</c:v>
+                  <c:v>8.236145973205566</c:v>
                 </c:pt>
                 <c:pt idx="36">
                   <c:v>0</c:v>
@@ -344,7 +344,7 @@
               <c:strCache>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-2aa6ce.o</c:v>
+                  <c:v>lto-llvm-30d3b0.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -464,112 +464,112 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>89.24064636230469</c:v>
+                  <c:v>90.54761505126953</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.432120800018311</c:v>
+                  <c:v>3.893737316131592</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8820575475692749</c:v>
+                  <c:v>0.7749112844467163</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.7292258143424988</c:v>
+                  <c:v>0.6406444907188416</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.5065280795097351</c:v>
+                  <c:v>0.444998562335968</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.4977948665618897</c:v>
+                  <c:v>0.4373261630535126</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.4846949875354767</c:v>
+                  <c:v>0.4258175790309906</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4060958027839661</c:v>
+                  <c:v>0.3567660748958588</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3842627108097076</c:v>
+                  <c:v>0.3375851213932037</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2707305252552033</c:v>
+                  <c:v>0.2378440648317337</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.240164190530777</c:v>
+                  <c:v>0.210990697145462</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2183310836553574</c:v>
+                  <c:v>0.1918097287416458</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1353652626276016</c:v>
+                  <c:v>0.1189220324158669</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.1222654059529305</c:v>
+                  <c:v>0.1074134483933449</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.1178987845778465</c:v>
+                  <c:v>0.1035772487521172</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1091655418276787</c:v>
+                  <c:v>0.09590486437082291</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.1091655418276787</c:v>
+                  <c:v>0.09590486437082291</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.1047989204525948</c:v>
+                  <c:v>0.09206866472959518</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.08733242750167847</c:v>
+                  <c:v>0.07672388851642609</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.08296580612659454</c:v>
+                  <c:v>0.07288769632577896</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.07859918475151062</c:v>
+                  <c:v>0.06905150413513184</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.07859918475151062</c:v>
+                  <c:v>0.06905150413513184</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.0742325633764267</c:v>
+                  <c:v>0.06521530449390411</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06986594200134277</c:v>
+                  <c:v>0.06137911230325699</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.06549932062625885</c:v>
+                  <c:v>0.05754291638731957</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.06549932062625885</c:v>
+                  <c:v>0.05754291638731957</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.06113270297646523</c:v>
+                  <c:v>0.05370672419667244</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.06113270297646523</c:v>
+                  <c:v>0.05370672419667244</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.06113270297646523</c:v>
+                  <c:v>0.05370672419667244</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.06113270297646523</c:v>
+                  <c:v>0.05370672419667244</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.0567660816013813</c:v>
+                  <c:v>0.04987052828073502</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.03929959237575531</c:v>
+                  <c:v>0.03452575206756592</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.02183310687541962</c:v>
+                  <c:v>0.01918097212910652</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.01746648550033569</c:v>
+                  <c:v>0.01534477807581425</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.01746648550033569</c:v>
+                  <c:v>0.01534477807581425</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.008733242750167847</c:v>
+                  <c:v>0.007672389037907124</c:v>
                 </c:pt>
                 <c:pt idx="36">
                   <c:v>0</c:v>
@@ -1036,25 +1036,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.75921630859375</v>
+        <v>91.76385498046875</v>
       </c>
       <c r="C3" s="1">
-        <v>11402</v>
+        <v>11409</v>
       </c>
       <c r="D3" s="1">
-        <v>40874</v>
+        <v>47207</v>
       </c>
       <c r="E3" s="1">
-        <v>40608</v>
+        <v>46940</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H3" s="1">
-        <v>11242</v>
+        <v>11248</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1062,7 +1062,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.240785598754883</v>
+        <v>8.236145973205566</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1169,25 +1169,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.24064636230469</v>
+        <v>90.54761505126953</v>
       </c>
       <c r="C3" s="1">
-        <v>40874</v>
+        <v>47207</v>
       </c>
       <c r="D3" s="1">
-        <v>11402</v>
+        <v>11409</v>
       </c>
       <c r="E3" s="1">
-        <v>40608</v>
+        <v>46940</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H3" s="1">
-        <v>11242</v>
+        <v>11248</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1195,7 +1195,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.432120800018311</v>
+        <v>3.893737316131592</v>
       </c>
       <c r="C4" s="1">
         <v>2030</v>
@@ -1221,7 +1221,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.8820575475692749</v>
+        <v>0.7749112844467163</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1247,7 +1247,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.7292258143424988</v>
+        <v>0.6406444907188416</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1273,7 +1273,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.5065280795097351</v>
+        <v>0.444998562335968</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1299,7 +1299,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.4977948665618897</v>
+        <v>0.4373261630535126</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1325,7 +1325,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.4846949875354767</v>
+        <v>0.4258175790309906</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1351,7 +1351,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.4060958027839661</v>
+        <v>0.3567660748958588</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1377,7 +1377,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.3842627108097076</v>
+        <v>0.3375851213932037</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1403,7 +1403,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2707305252552033</v>
+        <v>0.2378440648317337</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1429,7 +1429,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.240164190530777</v>
+        <v>0.210990697145462</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1455,7 +1455,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.2183310836553574</v>
+        <v>0.1918097287416458</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1481,7 +1481,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1353652626276016</v>
+        <v>0.1189220324158669</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1507,7 +1507,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.1222654059529305</v>
+        <v>0.1074134483933449</v>
       </c>
       <c r="C16" s="1">
         <v>56</v>
@@ -1533,7 +1533,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.1178987845778465</v>
+        <v>0.1035772487521172</v>
       </c>
       <c r="C17" s="1">
         <v>54</v>
@@ -1559,7 +1559,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.1091655418276787</v>
+        <v>0.09590486437082291</v>
       </c>
       <c r="C18" s="1">
         <v>50</v>
@@ -1585,7 +1585,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.1091655418276787</v>
+        <v>0.09590486437082291</v>
       </c>
       <c r="C19" s="1">
         <v>50</v>
@@ -1611,7 +1611,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.1047989204525948</v>
+        <v>0.09206866472959518</v>
       </c>
       <c r="C20" s="1">
         <v>48</v>
@@ -1637,7 +1637,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.08733242750167847</v>
+        <v>0.07672388851642609</v>
       </c>
       <c r="C21" s="1">
         <v>40</v>
@@ -1663,7 +1663,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.08296580612659454</v>
+        <v>0.07288769632577896</v>
       </c>
       <c r="C22" s="1">
         <v>38</v>
@@ -1689,7 +1689,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.07859918475151062</v>
+        <v>0.06905150413513184</v>
       </c>
       <c r="C23" s="1">
         <v>36</v>
@@ -1715,7 +1715,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.07859918475151062</v>
+        <v>0.06905150413513184</v>
       </c>
       <c r="C24" s="1">
         <v>36</v>
@@ -1741,7 +1741,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.0742325633764267</v>
+        <v>0.06521530449390411</v>
       </c>
       <c r="C25" s="1">
         <v>34</v>
@@ -1767,7 +1767,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06986594200134277</v>
+        <v>0.06137911230325699</v>
       </c>
       <c r="C26" s="1">
         <v>32</v>
@@ -1793,7 +1793,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.06549932062625885</v>
+        <v>0.05754291638731957</v>
       </c>
       <c r="C27" s="1">
         <v>30</v>
@@ -1819,7 +1819,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.06549932062625885</v>
+        <v>0.05754291638731957</v>
       </c>
       <c r="C28" s="1">
         <v>30</v>
@@ -1845,7 +1845,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.06113270297646523</v>
+        <v>0.05370672419667244</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1871,7 +1871,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.06113270297646523</v>
+        <v>0.05370672419667244</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1897,7 +1897,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.06113270297646523</v>
+        <v>0.05370672419667244</v>
       </c>
       <c r="C31" s="1">
         <v>28</v>
@@ -1923,7 +1923,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.06113270297646523</v>
+        <v>0.05370672419667244</v>
       </c>
       <c r="C32" s="1">
         <v>28</v>
@@ -1949,7 +1949,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.0567660816013813</v>
+        <v>0.04987052828073502</v>
       </c>
       <c r="C33" s="1">
         <v>26</v>
@@ -1975,7 +1975,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.03929959237575531</v>
+        <v>0.03452575206756592</v>
       </c>
       <c r="C34" s="1">
         <v>18</v>
@@ -2001,7 +2001,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.02183310687541962</v>
+        <v>0.01918097212910652</v>
       </c>
       <c r="C35" s="1">
         <v>10</v>
@@ -2027,7 +2027,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.01746648550033569</v>
+        <v>0.01534477807581425</v>
       </c>
       <c r="C36" s="1">
         <v>8</v>
@@ -2053,7 +2053,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="2">
-        <v>0.01746648550033569</v>
+        <v>0.01534477807581425</v>
       </c>
       <c r="C37" s="1">
         <v>8</v>
@@ -2079,7 +2079,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="2">
-        <v>0.008733242750167847</v>
+        <v>0.007672389037907124</v>
       </c>
       <c r="C38" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
add set temp and wind delay time
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -20,7 +20,7 @@
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-30d3b0.o</t>
+    <t>lto-llvm-06888a.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -249,7 +249,7 @@
               <c:strCache>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-30d3b0.o</c:v>
+                  <c:v>lto-llvm-06888a.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
@@ -267,10 +267,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>91.76385498046875</c:v>
+                  <c:v>91.76119995117188</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.236145973205566</c:v>
+                  <c:v>8.238796234130859</c:v>
                 </c:pt>
                 <c:pt idx="36">
                   <c:v>0</c:v>
@@ -344,7 +344,7 @@
               <c:strCache>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-30d3b0.o</c:v>
+                  <c:v>lto-llvm-06888a.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -464,112 +464,112 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="37"/>
                 <c:pt idx="0">
-                  <c:v>90.54761505126953</c:v>
+                  <c:v>89.27320098876953</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.893737316131592</c:v>
+                  <c:v>4.418711185455322</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.7749112844467163</c:v>
+                  <c:v>0.8793888092041016</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.6406444907188416</c:v>
+                  <c:v>0.7270194292068481</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.444998562335968</c:v>
+                  <c:v>0.5049955248832703</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.4373261630535126</c:v>
+                  <c:v>0.4962887167930603</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.4258175790309906</c:v>
+                  <c:v>0.483228474855423</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.3567660748958588</c:v>
+                  <c:v>0.4048671126365662</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3375851213932037</c:v>
+                  <c:v>0.3831000626087189</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2378440648317337</c:v>
+                  <c:v>0.2699114084243774</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.210990697145462</c:v>
+                  <c:v>0.239437535405159</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.1918097287416458</c:v>
+                  <c:v>0.2176704853773117</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1189220324158669</c:v>
+                  <c:v>0.1349557042121887</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.1074134483933449</c:v>
+                  <c:v>0.1218954771757126</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.1035772487521172</c:v>
+                  <c:v>0.117542065680027</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.09590486437082291</c:v>
+                  <c:v>0.1088352426886559</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.09590486437082291</c:v>
+                  <c:v>0.1088352426886559</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.09206866472959518</c:v>
+                  <c:v>0.1044818386435509</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.07672388851642609</c:v>
+                  <c:v>0.08706819266080856</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.07288769632577896</c:v>
+                  <c:v>0.08271478861570358</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.06905150413513184</c:v>
+                  <c:v>0.07836137712001801</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.06905150413513184</c:v>
+                  <c:v>0.07836137712001801</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.06521530449390411</c:v>
+                  <c:v>0.07400796562433243</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06137911230325699</c:v>
+                  <c:v>0.06965455412864685</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.05754291638731957</c:v>
+                  <c:v>0.06530115008354187</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.05754291638731957</c:v>
+                  <c:v>0.06530115008354187</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.05370672419667244</c:v>
+                  <c:v>0.06094773858785629</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.05370672419667244</c:v>
+                  <c:v>0.06094773858785629</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.05370672419667244</c:v>
+                  <c:v>0.06094773858785629</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.05370672419667244</c:v>
+                  <c:v>0.06094773858785629</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.04987052828073502</c:v>
+                  <c:v>0.05659432709217072</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.03452575206756592</c:v>
+                  <c:v>0.039180688560009</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.01918097212910652</c:v>
+                  <c:v>0.02176704816520214</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.01534477807581425</c:v>
+                  <c:v>0.01741363853216171</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.01534477807581425</c:v>
+                  <c:v>0.01741363853216171</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.007672389037907124</c:v>
+                  <c:v>0.008706819266080856</c:v>
                 </c:pt>
                 <c:pt idx="36">
                   <c:v>0</c:v>
@@ -1036,25 +1036,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.76385498046875</v>
+        <v>91.76119995117188</v>
       </c>
       <c r="C3" s="1">
-        <v>11409</v>
+        <v>11405</v>
       </c>
       <c r="D3" s="1">
-        <v>47207</v>
+        <v>41013</v>
       </c>
       <c r="E3" s="1">
-        <v>46940</v>
+        <v>40752</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11248</v>
+        <v>11250</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1062,7 +1062,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.236145973205566</v>
+        <v>8.238796234130859</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1169,25 +1169,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>90.54761505126953</v>
+        <v>89.27320098876953</v>
       </c>
       <c r="C3" s="1">
-        <v>47207</v>
+        <v>41013</v>
       </c>
       <c r="D3" s="1">
-        <v>11409</v>
+        <v>11405</v>
       </c>
       <c r="E3" s="1">
-        <v>46940</v>
+        <v>40752</v>
       </c>
       <c r="F3" s="1">
         <v>106</v>
       </c>
       <c r="G3" s="1">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11248</v>
+        <v>11250</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1195,7 +1195,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>3.893737316131592</v>
+        <v>4.418711185455322</v>
       </c>
       <c r="C4" s="1">
         <v>2030</v>
@@ -1221,7 +1221,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.7749112844467163</v>
+        <v>0.8793888092041016</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1247,7 +1247,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.6406444907188416</v>
+        <v>0.7270194292068481</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1273,7 +1273,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.444998562335968</v>
+        <v>0.5049955248832703</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1299,7 +1299,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.4373261630535126</v>
+        <v>0.4962887167930603</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1325,7 +1325,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.4258175790309906</v>
+        <v>0.483228474855423</v>
       </c>
       <c r="C9" s="1">
         <v>222</v>
@@ -1351,7 +1351,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.3567660748958588</v>
+        <v>0.4048671126365662</v>
       </c>
       <c r="C10" s="1">
         <v>186</v>
@@ -1377,7 +1377,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.3375851213932037</v>
+        <v>0.3831000626087189</v>
       </c>
       <c r="C11" s="1">
         <v>176</v>
@@ -1403,7 +1403,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2378440648317337</v>
+        <v>0.2699114084243774</v>
       </c>
       <c r="C12" s="1">
         <v>124</v>
@@ -1429,7 +1429,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.210990697145462</v>
+        <v>0.239437535405159</v>
       </c>
       <c r="C13" s="1">
         <v>110</v>
@@ -1455,7 +1455,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.1918097287416458</v>
+        <v>0.2176704853773117</v>
       </c>
       <c r="C14" s="1">
         <v>100</v>
@@ -1481,7 +1481,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1189220324158669</v>
+        <v>0.1349557042121887</v>
       </c>
       <c r="C15" s="1">
         <v>62</v>
@@ -1507,7 +1507,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.1074134483933449</v>
+        <v>0.1218954771757126</v>
       </c>
       <c r="C16" s="1">
         <v>56</v>
@@ -1533,7 +1533,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.1035772487521172</v>
+        <v>0.117542065680027</v>
       </c>
       <c r="C17" s="1">
         <v>54</v>
@@ -1559,7 +1559,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.09590486437082291</v>
+        <v>0.1088352426886559</v>
       </c>
       <c r="C18" s="1">
         <v>50</v>
@@ -1585,7 +1585,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.09590486437082291</v>
+        <v>0.1088352426886559</v>
       </c>
       <c r="C19" s="1">
         <v>50</v>
@@ -1611,7 +1611,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.09206866472959518</v>
+        <v>0.1044818386435509</v>
       </c>
       <c r="C20" s="1">
         <v>48</v>
@@ -1637,7 +1637,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.07672388851642609</v>
+        <v>0.08706819266080856</v>
       </c>
       <c r="C21" s="1">
         <v>40</v>
@@ -1663,7 +1663,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.07288769632577896</v>
+        <v>0.08271478861570358</v>
       </c>
       <c r="C22" s="1">
         <v>38</v>
@@ -1689,7 +1689,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.06905150413513184</v>
+        <v>0.07836137712001801</v>
       </c>
       <c r="C23" s="1">
         <v>36</v>
@@ -1715,7 +1715,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.06905150413513184</v>
+        <v>0.07836137712001801</v>
       </c>
       <c r="C24" s="1">
         <v>36</v>
@@ -1741,7 +1741,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.06521530449390411</v>
+        <v>0.07400796562433243</v>
       </c>
       <c r="C25" s="1">
         <v>34</v>
@@ -1767,7 +1767,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06137911230325699</v>
+        <v>0.06965455412864685</v>
       </c>
       <c r="C26" s="1">
         <v>32</v>
@@ -1793,7 +1793,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.05754291638731957</v>
+        <v>0.06530115008354187</v>
       </c>
       <c r="C27" s="1">
         <v>30</v>
@@ -1819,7 +1819,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.05754291638731957</v>
+        <v>0.06530115008354187</v>
       </c>
       <c r="C28" s="1">
         <v>30</v>
@@ -1845,7 +1845,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.05370672419667244</v>
+        <v>0.06094773858785629</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1871,7 +1871,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.05370672419667244</v>
+        <v>0.06094773858785629</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1897,7 +1897,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.05370672419667244</v>
+        <v>0.06094773858785629</v>
       </c>
       <c r="C31" s="1">
         <v>28</v>
@@ -1923,7 +1923,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.05370672419667244</v>
+        <v>0.06094773858785629</v>
       </c>
       <c r="C32" s="1">
         <v>28</v>
@@ -1949,7 +1949,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.04987052828073502</v>
+        <v>0.05659432709217072</v>
       </c>
       <c r="C33" s="1">
         <v>26</v>
@@ -1975,7 +1975,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.03452575206756592</v>
+        <v>0.039180688560009</v>
       </c>
       <c r="C34" s="1">
         <v>18</v>
@@ -2001,7 +2001,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.01918097212910652</v>
+        <v>0.02176704816520214</v>
       </c>
       <c r="C35" s="1">
         <v>10</v>
@@ -2027,7 +2027,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.01534477807581425</v>
+        <v>0.01741363853216171</v>
       </c>
       <c r="C36" s="1">
         <v>8</v>
@@ -2053,7 +2053,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="2">
-        <v>0.01534477807581425</v>
+        <v>0.01741363853216171</v>
       </c>
       <c r="C37" s="1">
         <v>8</v>
@@ -2079,7 +2079,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="2">
-        <v>0.007672389037907124</v>
+        <v>0.008706819266080856</v>
       </c>
       <c r="C38" s="1">
         <v>4</v>

</xml_diff>

<commit_message>
show quick countdown time when quick mode is running,software v1.4.4
</commit_message>
<xml_diff>
--- a/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
+++ b/app/project/MDK_V5/AT32F415RBT7_WorkBench_analysis.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
   <si>
     <t>AT32F415RBT7_WorkBench</t>
   </si>
   <si>
-    <t>lto-llvm-c66aaa.o</t>
+    <t>lto-llvm-d8ae17.o</t>
   </si>
   <si>
     <t>startup_at32f415.o</t>
@@ -38,16 +38,10 @@
     <t>dmul.o</t>
   </si>
   <si>
-    <t>ddiv.o</t>
-  </si>
-  <si>
     <t>depilogue.o</t>
   </si>
   <si>
     <t>fadd.o</t>
-  </si>
-  <si>
-    <t>fdiv.o</t>
   </si>
   <si>
     <t>fepilogue.o</t>
@@ -245,16 +239,16 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>ram_percent!$A$3:$A$39</c:f>
+              <c:f>ram_percent!$A$3:$A$37</c:f>
               <c:strCache>
-                <c:ptCount val="37"/>
+                <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-c66aaa.o</c:v>
+                  <c:v>lto-llvm-d8ae17.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>startup_at32f415.o</c:v>
                 </c:pt>
-                <c:pt idx="36">
+                <c:pt idx="34">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -262,17 +256,17 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>ram_percent!$B$3:$B$39</c:f>
+              <c:f>ram_percent!$B$3:$B$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="37"/>
+                <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>91.76119995117188</c:v>
+                  <c:v>91.76518249511719</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.238796234130859</c:v>
-                </c:pt>
-                <c:pt idx="36">
+                  <c:v>8.234821319580078</c:v>
+                </c:pt>
+                <c:pt idx="34">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -340,11 +334,11 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>flash_percent!$A$3:$A$39</c:f>
+              <c:f>flash_percent!$A$3:$A$37</c:f>
               <c:strCache>
-                <c:ptCount val="37"/>
+                <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>lto-llvm-c66aaa.o</c:v>
+                  <c:v>lto-llvm-d8ae17.o</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>mf_w.l</c:v>
@@ -362,96 +356,90 @@
                   <c:v>dmul.o</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>ddiv.o</c:v>
+                  <c:v>depilogue.o</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>depilogue.o</c:v>
+                  <c:v>fadd.o</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>fadd.o</c:v>
+                  <c:v>fepilogue.o</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>fdiv.o</c:v>
+                  <c:v>fmul.o</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>fepilogue.o</c:v>
+                  <c:v>dfixi.o</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>fmul.o</c:v>
+                  <c:v>d2f.o</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>dfixi.o</c:v>
+                  <c:v>dcmpgt.o</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>d2f.o</c:v>
+                  <c:v>ffixi.o</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>dcmpgt.o</c:v>
+                  <c:v>dfixui.o</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>ffixi.o</c:v>
+                  <c:v>init.o</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>dfixui.o</c:v>
+                  <c:v>ffixui.o</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>init.o</c:v>
+                  <c:v>f2d.o</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>ffixui.o</c:v>
+                  <c:v>memseta.o</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>f2d.o</c:v>
+                  <c:v>llsshr.o</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>memseta.o</c:v>
+                  <c:v>dflti.o</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>llsshr.o</c:v>
+                  <c:v>llushr.o</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>dflti.o</c:v>
+                  <c:v>llshl.o</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>llushr.o</c:v>
+                  <c:v>handlers.o</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>llshl.o</c:v>
+                  <c:v>fcmplt.o</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>handlers.o</c:v>
+                  <c:v>fcmple.o</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>fcmplt.o</c:v>
+                  <c:v>fcmpgt.o</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>fcmple.o</c:v>
+                  <c:v>fcmpge.o</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>fcmpgt.o</c:v>
+                  <c:v>dfltui.o</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>fcmpge.o</c:v>
+                  <c:v>fflti.o</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>dfltui.o</c:v>
+                  <c:v>ffltui.o</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>fflti.o</c:v>
+                  <c:v>entry9a.o</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>ffltui.o</c:v>
+                  <c:v>entry2.o</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>entry9a.o</c:v>
+                  <c:v>entry5.o</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>entry2.o</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>entry5.o</c:v>
-                </c:pt>
-                <c:pt idx="36">
                   <c:v>Totals</c:v>
                 </c:pt>
               </c:strCache>
@@ -459,119 +447,113 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>flash_percent!$B$3:$B$39</c:f>
+              <c:f>flash_percent!$B$3:$B$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="37"/>
+                <c:ptCount val="35"/>
                 <c:pt idx="0">
-                  <c:v>89.27320098876953</c:v>
+                  <c:v>93.97653961181641</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.418711185455322</c:v>
+                  <c:v>2.394596576690674</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8793888092041016</c:v>
+                  <c:v>0.5744756460189819</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.7270194292068481</c:v>
+                  <c:v>0.4749377965927124</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.5049955248832703</c:v>
+                  <c:v>0.3298968970775604</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.4962887167930603</c:v>
+                  <c:v>0.3242090344429016</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.483228474855423</c:v>
+                  <c:v>0.2644863128662109</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4048671126365662</c:v>
+                  <c:v>0.2502666115760803</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3831000626087189</c:v>
+                  <c:v>0.1564166396856308</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2699114084243774</c:v>
+                  <c:v>0.1421969383955002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.239437535405159</c:v>
+                  <c:v>0.08816210180521011</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2176704853773117</c:v>
+                  <c:v>0.0796302855014801</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.1349557042121887</c:v>
+                  <c:v>0.0767863467335701</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.1218954771757126</c:v>
+                  <c:v>0.07109846919775009</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.117542065680027</c:v>
+                  <c:v>0.07109846919775009</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.1088352426886559</c:v>
+                  <c:v>0.06825453042984009</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.1088352426886559</c:v>
+                  <c:v>0.05687877535820007</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.1044818386435509</c:v>
+                  <c:v>0.05403483659029007</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.08706819266080856</c:v>
+                  <c:v>0.05119089782238007</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.08271478861570358</c:v>
+                  <c:v>0.05119089782238007</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.07836137712001801</c:v>
+                  <c:v>0.04834695905447006</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.07836137712001801</c:v>
+                  <c:v>0.04550302028656006</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.07400796562433243</c:v>
+                  <c:v>0.04265908151865006</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.06965455412864685</c:v>
+                  <c:v>0.04265908151865006</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.06530115008354187</c:v>
+                  <c:v>0.03981514275074005</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.06530115008354187</c:v>
+                  <c:v>0.03981514275074005</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.06094773858785629</c:v>
+                  <c:v>0.03981514275074005</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.06094773858785629</c:v>
+                  <c:v>0.03981514275074005</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.06094773858785629</c:v>
+                  <c:v>0.03697120398283005</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.06094773858785629</c:v>
+                  <c:v>0.02559544891119003</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.05659432709217072</c:v>
+                  <c:v>0.01421969383955002</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.039180688560009</c:v>
+                  <c:v>0.01137575507164002</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.02176704816520214</c:v>
+                  <c:v>0.01137575507164002</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.01741363853216171</c:v>
+                  <c:v>0.005687877535820007</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.01741363853216171</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>0.008706819266080856</c:v>
-                </c:pt>
-                <c:pt idx="36">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -676,8 +658,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H39" totalsRowCount="1">
-  <autoFilter ref="A2:H38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A2:H37" totalsRowCount="1">
+  <autoFilter ref="A2:H36"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="ram_percent" totalsRowFunction="sum"/>
@@ -693,8 +675,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H39" totalsRowCount="1">
-  <autoFilter ref="A2:H38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A2:H37" totalsRowCount="1">
+  <autoFilter ref="A2:H36"/>
   <tableColumns count="8">
     <tableColumn id="1" name="File_name" totalsRowLabel="Totals"/>
     <tableColumn id="2" name="flash_percent" totalsRowFunction="sum"/>
@@ -994,7 +976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1007,28 +989,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
         <v>37</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>40</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>41</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>42</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>43</v>
-      </c>
-      <c r="G2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1036,25 +1018,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>91.76119995117188</v>
+        <v>91.76518249511719</v>
       </c>
       <c r="C3" s="1">
-        <v>11405</v>
+        <v>11411</v>
       </c>
       <c r="D3" s="1">
-        <v>41013</v>
+        <v>66089</v>
       </c>
       <c r="E3" s="1">
-        <v>40752</v>
+        <v>65844</v>
       </c>
       <c r="F3" s="1">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="G3" s="1">
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11250</v>
+        <v>11256</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1062,7 +1044,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>8.238796234130859</v>
+        <v>8.234821319580078</v>
       </c>
       <c r="C4" s="1">
         <v>1024</v>
@@ -1083,35 +1065,35 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39">
+    <row r="37" spans="1:8">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
         <f>SUBTOTAL(109,[ram_percent])</f>
         <v>0</v>
       </c>
-      <c r="C39">
+      <c r="C37">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="D39">
+      <c r="D37">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="E39">
+      <c r="E37">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F39">
+      <c r="F37">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G39">
+      <c r="G37">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H39">
+      <c r="H37">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>
@@ -1127,7 +1109,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="16.7109375" customWidth="1"/>
@@ -1140,28 +1122,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" t="s">
         <v>41</v>
       </c>
-      <c r="D2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>42</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>43</v>
-      </c>
-      <c r="G2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1169,25 +1151,25 @@
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>89.27320098876953</v>
+        <v>93.97653961181641</v>
       </c>
       <c r="C3" s="1">
-        <v>41013</v>
+        <v>66089</v>
       </c>
       <c r="D3" s="1">
-        <v>11405</v>
+        <v>11411</v>
       </c>
       <c r="E3" s="1">
-        <v>40752</v>
+        <v>65844</v>
       </c>
       <c r="F3" s="1">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="G3" s="1">
         <v>155</v>
       </c>
       <c r="H3" s="1">
-        <v>11250</v>
+        <v>11256</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1195,16 +1177,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>4.418711185455322</v>
+        <v>2.394596576690674</v>
       </c>
       <c r="C4" s="1">
-        <v>2030</v>
+        <v>1684</v>
       </c>
       <c r="D4" s="1">
         <v>0</v>
       </c>
       <c r="E4" s="1">
-        <v>2030</v>
+        <v>1684</v>
       </c>
       <c r="F4" s="1">
         <v>0</v>
@@ -1221,7 +1203,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2">
-        <v>0.8793888092041016</v>
+        <v>0.5744756460189819</v>
       </c>
       <c r="C5" s="1">
         <v>404</v>
@@ -1247,7 +1229,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0.7270194292068481</v>
+        <v>0.4749377965927124</v>
       </c>
       <c r="C6" s="1">
         <v>334</v>
@@ -1273,7 +1255,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
-        <v>0.5049955248832703</v>
+        <v>0.3298968970775604</v>
       </c>
       <c r="C7" s="1">
         <v>232</v>
@@ -1299,7 +1281,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>0.4962887167930603</v>
+        <v>0.3242090344429016</v>
       </c>
       <c r="C8" s="1">
         <v>228</v>
@@ -1325,16 +1307,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
-        <v>0.483228474855423</v>
+        <v>0.2644863128662109</v>
       </c>
       <c r="C9" s="1">
-        <v>222</v>
+        <v>186</v>
       </c>
       <c r="D9" s="1">
         <v>0</v>
       </c>
       <c r="E9" s="1">
-        <v>222</v>
+        <v>186</v>
       </c>
       <c r="F9" s="1">
         <v>0</v>
@@ -1351,16 +1333,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
-        <v>0.4048671126365662</v>
+        <v>0.2502666115760803</v>
       </c>
       <c r="C10" s="1">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="D10" s="1">
         <v>0</v>
       </c>
       <c r="E10" s="1">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="F10" s="1">
         <v>0</v>
@@ -1377,16 +1359,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
-        <v>0.3831000626087189</v>
+        <v>0.1564166396856308</v>
       </c>
       <c r="C11" s="1">
-        <v>176</v>
+        <v>110</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
       </c>
       <c r="E11" s="1">
-        <v>176</v>
+        <v>110</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
@@ -1403,16 +1385,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2699114084243774</v>
+        <v>0.1421969383955002</v>
       </c>
       <c r="C12" s="1">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="D12" s="1">
         <v>0</v>
       </c>
       <c r="E12" s="1">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="F12" s="1">
         <v>0</v>
@@ -1429,16 +1411,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
-        <v>0.239437535405159</v>
+        <v>0.08816210180521011</v>
       </c>
       <c r="C13" s="1">
-        <v>110</v>
+        <v>62</v>
       </c>
       <c r="D13" s="1">
         <v>0</v>
       </c>
       <c r="E13" s="1">
-        <v>110</v>
+        <v>62</v>
       </c>
       <c r="F13" s="1">
         <v>0</v>
@@ -1455,16 +1437,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
-        <v>0.2176704853773117</v>
+        <v>0.0796302855014801</v>
       </c>
       <c r="C14" s="1">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="D14" s="1">
         <v>0</v>
       </c>
       <c r="E14" s="1">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
@@ -1481,16 +1463,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
-        <v>0.1349557042121887</v>
+        <v>0.0767863467335701</v>
       </c>
       <c r="C15" s="1">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D15" s="1">
         <v>0</v>
       </c>
       <c r="E15" s="1">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="F15" s="1">
         <v>0</v>
@@ -1507,16 +1489,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>0.1218954771757126</v>
+        <v>0.07109846919775009</v>
       </c>
       <c r="C16" s="1">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -1533,16 +1515,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="2">
-        <v>0.117542065680027</v>
+        <v>0.07109846919775009</v>
       </c>
       <c r="C17" s="1">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D17" s="1">
         <v>0</v>
       </c>
       <c r="E17" s="1">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F17" s="1">
         <v>0</v>
@@ -1559,16 +1541,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="2">
-        <v>0.1088352426886559</v>
+        <v>0.06825453042984009</v>
       </c>
       <c r="C18" s="1">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -1585,16 +1567,16 @@
         <v>17</v>
       </c>
       <c r="B19" s="2">
-        <v>0.1088352426886559</v>
+        <v>0.05687877535820007</v>
       </c>
       <c r="C19" s="1">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D19" s="1">
         <v>0</v>
       </c>
       <c r="E19" s="1">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
@@ -1611,16 +1593,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="2">
-        <v>0.1044818386435509</v>
+        <v>0.05403483659029007</v>
       </c>
       <c r="C20" s="1">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
@@ -1637,16 +1619,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="2">
-        <v>0.08706819266080856</v>
+        <v>0.05119089782238007</v>
       </c>
       <c r="C21" s="1">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D21" s="1">
         <v>0</v>
       </c>
       <c r="E21" s="1">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F21" s="1">
         <v>0</v>
@@ -1663,16 +1645,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="2">
-        <v>0.08271478861570358</v>
+        <v>0.05119089782238007</v>
       </c>
       <c r="C22" s="1">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D22" s="1">
         <v>0</v>
       </c>
       <c r="E22" s="1">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F22" s="1">
         <v>0</v>
@@ -1689,16 +1671,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="2">
-        <v>0.07836137712001801</v>
+        <v>0.04834695905447006</v>
       </c>
       <c r="C23" s="1">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D23" s="1">
         <v>0</v>
       </c>
       <c r="E23" s="1">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F23" s="1">
         <v>0</v>
@@ -1715,16 +1697,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>0.07836137712001801</v>
+        <v>0.04550302028656006</v>
       </c>
       <c r="C24" s="1">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D24" s="1">
         <v>0</v>
       </c>
       <c r="E24" s="1">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F24" s="1">
         <v>0</v>
@@ -1741,16 +1723,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.07400796562433243</v>
+        <v>0.04265908151865006</v>
       </c>
       <c r="C25" s="1">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -1767,16 +1749,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>0.06965455412864685</v>
+        <v>0.04265908151865006</v>
       </c>
       <c r="C26" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D26" s="1">
         <v>0</v>
       </c>
       <c r="E26" s="1">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F26" s="1">
         <v>0</v>
@@ -1793,16 +1775,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="2">
-        <v>0.06530115008354187</v>
+        <v>0.03981514275074005</v>
       </c>
       <c r="C27" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D27" s="1">
         <v>0</v>
       </c>
       <c r="E27" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F27" s="1">
         <v>0</v>
@@ -1819,16 +1801,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="2">
-        <v>0.06530115008354187</v>
+        <v>0.03981514275074005</v>
       </c>
       <c r="C28" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D28" s="1">
         <v>0</v>
       </c>
       <c r="E28" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F28" s="1">
         <v>0</v>
@@ -1845,7 +1827,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>0.06094773858785629</v>
+        <v>0.03981514275074005</v>
       </c>
       <c r="C29" s="1">
         <v>28</v>
@@ -1871,7 +1853,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>0.06094773858785629</v>
+        <v>0.03981514275074005</v>
       </c>
       <c r="C30" s="1">
         <v>28</v>
@@ -1897,16 +1879,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>0.06094773858785629</v>
+        <v>0.03697120398283005</v>
       </c>
       <c r="C31" s="1">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D31" s="1">
         <v>0</v>
       </c>
       <c r="E31" s="1">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F31" s="1">
         <v>0</v>
@@ -1923,16 +1905,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>0.06094773858785629</v>
+        <v>0.02559544891119003</v>
       </c>
       <c r="C32" s="1">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D32" s="1">
         <v>0</v>
       </c>
       <c r="E32" s="1">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F32" s="1">
         <v>0</v>
@@ -1949,16 +1931,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>0.05659432709217072</v>
+        <v>0.01421969383955002</v>
       </c>
       <c r="C33" s="1">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="D33" s="1">
         <v>0</v>
       </c>
       <c r="E33" s="1">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
@@ -1975,16 +1957,16 @@
         <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>0.039180688560009</v>
+        <v>0.01137575507164002</v>
       </c>
       <c r="C34" s="1">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D34" s="1">
         <v>0</v>
       </c>
       <c r="E34" s="1">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F34" s="1">
         <v>0</v>
@@ -2001,16 +1983,16 @@
         <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>0.02176704816520214</v>
+        <v>0.01137575507164002</v>
       </c>
       <c r="C35" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D35" s="1">
         <v>0</v>
       </c>
       <c r="E35" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F35" s="1">
         <v>0</v>
@@ -2027,16 +2009,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>0.01741363853216171</v>
+        <v>0.005687877535820007</v>
       </c>
       <c r="C36" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D36" s="1">
         <v>0</v>
       </c>
       <c r="E36" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F36" s="1">
         <v>0</v>
@@ -2049,86 +2031,34 @@
       </c>
     </row>
     <row r="37" spans="1:8">
-      <c r="A37" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B37" s="2">
-        <v>0.01741363853216171</v>
-      </c>
-      <c r="C37" s="1">
-        <v>8</v>
-      </c>
-      <c r="D37" s="1">
-        <v>0</v>
-      </c>
-      <c r="E37" s="1">
-        <v>8</v>
-      </c>
-      <c r="F37" s="1">
-        <v>0</v>
-      </c>
-      <c r="G37" s="1">
-        <v>0</v>
-      </c>
-      <c r="H37" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="1" t="s">
+      <c r="A37" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="2">
-        <v>0.008706819266080856</v>
-      </c>
-      <c r="C38" s="1">
-        <v>4</v>
-      </c>
-      <c r="D38" s="1">
-        <v>0</v>
-      </c>
-      <c r="E38" s="1">
-        <v>4</v>
-      </c>
-      <c r="F38" s="1">
-        <v>0</v>
-      </c>
-      <c r="G38" s="1">
-        <v>0</v>
-      </c>
-      <c r="H38" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39">
+      <c r="B37">
         <f>SUBTOTAL(109,[flash_percent])</f>
         <v>0</v>
       </c>
-      <c r="C39">
+      <c r="C37">
         <f>SUBTOTAL(109,[flash])</f>
         <v>0</v>
       </c>
-      <c r="D39">
+      <c r="D37">
         <f>SUBTOTAL(109,[ram])</f>
         <v>0</v>
       </c>
-      <c r="E39">
+      <c r="E37">
         <f>SUBTOTAL(109,[Code])</f>
         <v>0</v>
       </c>
-      <c r="F39">
+      <c r="F37">
         <f>SUBTOTAL(109,[RO_data])</f>
         <v>0</v>
       </c>
-      <c r="G39">
+      <c r="G37">
         <f>SUBTOTAL(109,[RW_data])</f>
         <v>0</v>
       </c>
-      <c r="H39">
+      <c r="H37">
         <f>SUBTOTAL(109,[ZI_data])</f>
         <v>0</v>
       </c>

</xml_diff>